<commit_message>
client changes on 31 aug 2026
</commit_message>
<xml_diff>
--- a/src/server/data/contacts.xlsx
+++ b/src/server/data/contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -565,9 +565,35 @@
         <v>31 Aug 2026, 11:41:17 am</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>test1</v>
+      </c>
+      <c r="C7" t="str">
+        <v>test</v>
+      </c>
+      <c r="D7" t="str">
+        <v>test@gmail.com</v>
+      </c>
+      <c r="E7" t="str">
+        <v>9876543219</v>
+      </c>
+      <c r="F7" t="str">
+        <v>test@1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>test @test @ test</v>
+      </c>
+      <c r="H7" t="str">
+        <v>31 Aug 2026, 12:39:08 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>